<commit_message>
thay doi cau truc folder sau khi bi lit pha huy
</commit_message>
<xml_diff>
--- a/Zzz_data/LMDO data_3i/depots_vietnam.xlsx
+++ b/Zzz_data/LMDO data_3i/depots_vietnam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\A UEH_UNIVERSITY\UEH_Subjects\LMDO\Lastmile\Zzz_data\LMDO data_3i\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B41E482-5E6D-4251-8F17-FC09BB6AFE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960E3840-49E7-4B37-9099-A95BEC564D34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -589,16 +589,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.1796875" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15.453125" customWidth="1"/>
-    <col min="5" max="5" width="16.90625" customWidth="1"/>
-    <col min="6" max="6" width="20.90625" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" customWidth="1"/>
+    <col min="6" max="6" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -618,7 +618,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -638,7 +638,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -658,7 +658,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -678,7 +678,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -698,7 +698,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -718,7 +718,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -738,7 +738,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -758,7 +758,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -778,7 +778,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -798,7 +798,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -818,7 +818,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -838,7 +838,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -858,7 +858,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -878,7 +878,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -898,7 +898,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -918,7 +918,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -938,7 +938,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -958,7 +958,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -978,7 +978,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -998,7 +998,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>55</v>
       </c>

</xml_diff>